<commit_message>
feat: remove location and preference from the match score
Location proximity and work-type/arrangement preference are no longer
scored components — they only drive the Jobs page's location filter
(rec.location.level / matchesLocation). Their former 15 + 10 points
are folded proportionally into skills/suitability/education
(35/25/15 -> 47/33/20, still summing to 100), so the "how the score
is built" breakdown and info panel now list every factor the score
actually uses. Regenerates the thesis dataset exports and retrains
the Decision Tree on the resulting 3-feature set.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ml/output/training_report.xlsx
+++ b/ml/output/training_report.xlsx
@@ -484,7 +484,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>64.8%</t>
+          <t>41.8%</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -536,23 +536,23 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.6342028831999499</v>
+        <v>0.6472109520194749</v>
       </c>
       <c r="C2" t="n">
-        <v>0.4222676613918383</v>
+        <v>0.567655100227593</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Job-type &amp; work-setup preference</t>
+          <t>Skill coverage</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.2299608937269878</v>
+        <v>0.3527890479805252</v>
       </c>
       <c r="C3" t="n">
-        <v>0.170735076019459</v>
+        <v>0.36476922798491</v>
       </c>
     </row>
     <row r="4">
@@ -562,48 +562,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.1024613147696201</v>
+        <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1919579736074057</v>
+        <v>0.06757567178749699</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Skill coverage</t>
+          <t>Disability type explicitly listed</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.0314908408992156</v>
+        <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>0.1222425765409031</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Location proximity</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>0.001884067404226521</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0.09279671244039389</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Disability type explicitly listed</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -645,7 +619,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.8695652173913043</v>
+        <v>1</v>
       </c>
       <c r="C2" t="n">
         <v>1</v>
@@ -658,7 +632,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.875</v>
+        <v>1</v>
       </c>
       <c r="C3" t="n">
         <v>1</v>
@@ -671,7 +645,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.9333333333333333</v>
+        <v>1</v>
       </c>
       <c r="C4" t="n">
         <v>1</v>
@@ -684,7 +658,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.9032258064516129</v>
+        <v>1</v>
       </c>
       <c r="C5" t="n">
         <v>1</v>
@@ -723,10 +697,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="C2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -736,10 +710,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C3" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -785,16 +759,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.8571428571428571</v>
+        <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3">
@@ -804,16 +778,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.875</v>
+        <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>0.9333333333333333</v>
+        <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>0.9032258064516129</v>
+        <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4">
@@ -823,16 +797,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.8695652173913043</v>
+        <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>0.8695652173913043</v>
+        <v>1</v>
       </c>
       <c r="D4" t="n">
-        <v>0.8695652173913043</v>
+        <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>0.8695652173913043</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -842,13 +816,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.8660714285714286</v>
+        <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>0.8416666666666667</v>
+        <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>0.8516129032258064</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
         <v>23</v>
@@ -861,13 +835,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.8687888198757764</v>
+        <v>1</v>
       </c>
       <c r="C6" t="n">
-        <v>0.8695652173913043</v>
+        <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>0.8673211781206172</v>
+        <v>1</v>
       </c>
       <c r="E6" t="n">
         <v>23</v>
@@ -884,7 +858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -915,30 +889,20 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>location_fraction</t>
+          <t>disability_listed</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>preference_fraction</t>
+          <t>actual_label</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>disability_listed</t>
+          <t>predicted_label</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>actual_label</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>predicted_label</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>correct</t>
         </is>
@@ -947,51 +911,45 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PWD-LB-2024-0042</t>
+          <t>PWD-LB-2024-0044</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>JOB-003</t>
+          <t>JOB-008</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.35</v>
+        <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>0.91</v>
+        <v>0.21</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
         <v>1</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K2" t="b">
+        <v>1</v>
+      </c>
+      <c r="I2" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PWD-LB-2024-0045</t>
+          <t>PWD-LB-2024-0044</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>JOB-005</t>
+          <t>JOB-011</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -1001,40 +959,34 @@
         <v>0.21</v>
       </c>
       <c r="E3" t="n">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>0.35</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
       </c>
-      <c r="I3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" t="n">
-        <v>1</v>
-      </c>
-      <c r="K3" t="b">
-        <v>0</v>
+      <c r="I3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PWD-LB-2024-0043</t>
+          <t>PWD-LB-2024-0046</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>JOB-004</t>
+          <t>JOB-012</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.75</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
         <v>0.91</v>
@@ -1043,21 +995,15 @@
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K4" t="b">
+        <v>1</v>
+      </c>
+      <c r="I4" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1069,11 +1015,11 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>JOB-006</t>
+          <t>JOB-001</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D5" t="n">
         <v>0.21</v>
@@ -1082,37 +1028,31 @@
         <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>0.35</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
       </c>
-      <c r="I5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="b">
+      <c r="I5" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PWD-LB-2024-0044</t>
+          <t>PWD-LB-2024-0043</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>JOB-005</t>
+          <t>JOB-009</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D6" t="n">
         <v>0.21</v>
@@ -1121,72 +1061,60 @@
         <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>0.35</v>
+        <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
       </c>
-      <c r="I6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="b">
+      <c r="I6" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PWD-LB-2024-0048</t>
+          <t>PWD-LB-2024-0042</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>JOB-006</t>
+          <t>JOB-004</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1</v>
+        <v>0.85</v>
       </c>
       <c r="D7" t="n">
-        <v>0.21</v>
+        <v>0.4433</v>
       </c>
       <c r="E7" t="n">
         <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>0.35</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
         <v>1</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J7" t="n">
-        <v>1</v>
-      </c>
-      <c r="K7" t="b">
+        <v>1</v>
+      </c>
+      <c r="I7" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PWD-LB-2024-0047</t>
+          <t>PWD-LB-2024-0045</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>JOB-011</t>
+          <t>JOB-004</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1196,274 +1124,232 @@
         <v>0.21</v>
       </c>
       <c r="E8" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="F8" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
       </c>
-      <c r="I8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" t="b">
+      <c r="I8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>PWD-LB-2024-0048</t>
+          <t>PWD-LB-2024-0043</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>JOB-005</t>
+          <t>JOB-007</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.75</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="D9" t="n">
-        <v>0.21</v>
+        <v>0.91</v>
       </c>
       <c r="E9" t="n">
         <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>0.35</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
         <v>1</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" t="n">
-        <v>1</v>
-      </c>
-      <c r="J9" t="n">
-        <v>1</v>
-      </c>
-      <c r="K9" t="b">
+        <v>1</v>
+      </c>
+      <c r="I9" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>PWD-LB-2024-0044</t>
+          <t>PWD-LB-2024-0045</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>JOB-012</t>
+          <t>JOB-009</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D10" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.91</v>
       </c>
       <c r="E10" t="n">
         <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" t="n">
-        <v>1</v>
-      </c>
-      <c r="J10" t="n">
-        <v>1</v>
-      </c>
-      <c r="K10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I10" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PWD-LB-2024-0043</t>
+          <t>PWD-LB-2024-0047</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>JOB-006</t>
+          <t>JOB-007</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>0.91</v>
+        <v>0.21</v>
       </c>
       <c r="E11" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="F11" t="n">
-        <v>0.35</v>
+        <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
       </c>
-      <c r="I11" t="n">
-        <v>1</v>
-      </c>
-      <c r="J11" t="n">
-        <v>1</v>
-      </c>
-      <c r="K11" t="b">
+      <c r="I11" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PWD-LB-2024-0047</t>
+          <t>PWD-LB-2024-0042</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>JOB-008</t>
+          <t>JOB-002</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.7</v>
+        <v>0.48</v>
       </c>
       <c r="D12" t="n">
-        <v>0.21</v>
+        <v>0.4433</v>
       </c>
       <c r="E12" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H12" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" t="n">
-        <v>1</v>
-      </c>
-      <c r="J12" t="n">
-        <v>0</v>
-      </c>
-      <c r="K12" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="I12" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>PWD-LB-2024-0043</t>
+          <t>PWD-LB-2024-0042</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>JOB-003</t>
+          <t>JOB-007</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="D13" t="n">
-        <v>0.91</v>
+        <v>0.4433</v>
       </c>
       <c r="E13" t="n">
         <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" t="n">
-        <v>1</v>
-      </c>
-      <c r="J13" t="n">
-        <v>1</v>
-      </c>
-      <c r="K13" t="b">
+        <v>1</v>
+      </c>
+      <c r="I13" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PWD-LB-2024-0042</t>
+          <t>PWD-LB-2024-0045</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>JOB-009</t>
+          <t>JOB-011</t>
         </is>
       </c>
       <c r="C14" t="n">
         <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>0.21</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="E14" t="n">
         <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
       </c>
-      <c r="I14" t="n">
-        <v>1</v>
-      </c>
-      <c r="J14" t="n">
-        <v>1</v>
-      </c>
-      <c r="K14" t="b">
+      <c r="I14" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PWD-LB-2024-0046</t>
+          <t>PWD-LB-2024-0047</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>JOB-009</t>
+          <t>JOB-013</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D15" t="n">
         <v>0.91</v>
@@ -1472,21 +1358,15 @@
         <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H15" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" t="n">
-        <v>1</v>
-      </c>
-      <c r="J15" t="n">
-        <v>1</v>
-      </c>
-      <c r="K15" t="b">
+        <v>1</v>
+      </c>
+      <c r="I15" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1498,254 +1378,218 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>JOB-001</t>
+          <t>JOB-003</t>
         </is>
       </c>
       <c r="C16" t="n">
         <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>0.21</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="E16" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="F16" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
       </c>
-      <c r="I16" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" t="n">
-        <v>1</v>
-      </c>
-      <c r="K16" t="b">
-        <v>0</v>
+      <c r="I16" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>PWD-LB-2024-0047</t>
+          <t>PWD-LB-2024-0044</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>JOB-010</t>
+          <t>JOB-003</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="D17" t="n">
-        <v>0.91</v>
+        <v>0.21</v>
       </c>
       <c r="E17" t="n">
         <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G17" t="n">
         <v>1</v>
       </c>
       <c r="H17" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" t="n">
-        <v>1</v>
-      </c>
-      <c r="J17" t="n">
-        <v>1</v>
-      </c>
-      <c r="K17" t="b">
+        <v>1</v>
+      </c>
+      <c r="I17" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>PWD-LB-2024-0043</t>
+          <t>PWD-LB-2024-0048</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>JOB-011</t>
+          <t>JOB-012</t>
         </is>
       </c>
       <c r="C18" t="n">
         <v>0</v>
       </c>
       <c r="D18" t="n">
-        <v>0.91</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="E18" t="n">
         <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H18" t="n">
         <v>0</v>
       </c>
-      <c r="I18" t="n">
-        <v>1</v>
-      </c>
-      <c r="J18" t="n">
-        <v>1</v>
-      </c>
-      <c r="K18" t="b">
+      <c r="I18" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>PWD-LB-2024-0047</t>
+          <t>PWD-LB-2024-0048</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>JOB-005</t>
+          <t>JOB-013</t>
         </is>
       </c>
       <c r="C19" t="n">
         <v>0</v>
       </c>
       <c r="D19" t="n">
-        <v>0.21</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="E19" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>0.35</v>
+        <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H19" t="n">
         <v>0</v>
       </c>
-      <c r="I19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K19" t="b">
+      <c r="I19" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>PWD-LB-2024-0042</t>
+          <t>PWD-LB-2024-0047</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>JOB-007</t>
+          <t>JOB-003</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="D20" t="n">
-        <v>0.4433</v>
+        <v>0.21</v>
       </c>
       <c r="E20" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="F20" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H20" t="n">
         <v>0</v>
       </c>
-      <c r="I20" t="n">
-        <v>1</v>
-      </c>
-      <c r="J20" t="n">
-        <v>1</v>
-      </c>
-      <c r="K20" t="b">
+      <c r="I20" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>PWD-LB-2024-0046</t>
+          <t>PWD-LB-2024-0044</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>JOB-011</t>
+          <t>JOB-006</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="D21" t="n">
-        <v>0.91</v>
+        <v>0.21</v>
       </c>
       <c r="E21" t="n">
         <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H21" t="n">
         <v>0</v>
       </c>
-      <c r="I21" t="n">
-        <v>1</v>
-      </c>
-      <c r="J21" t="n">
-        <v>1</v>
-      </c>
-      <c r="K21" t="b">
+      <c r="I21" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>PWD-LB-2024-0046</t>
+          <t>PWD-LB-2024-0048</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>JOB-004</t>
+          <t>JOB-009</t>
         </is>
       </c>
       <c r="C22" t="n">
         <v>0</v>
       </c>
       <c r="D22" t="n">
-        <v>0.21</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="E22" t="n">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="F22" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G22" t="n">
         <v>0</v>
@@ -1753,20 +1597,14 @@
       <c r="H22" t="n">
         <v>0</v>
       </c>
-      <c r="I22" t="n">
-        <v>0</v>
-      </c>
-      <c r="J22" t="n">
-        <v>0</v>
-      </c>
-      <c r="K22" t="b">
+      <c r="I22" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>PWD-LB-2024-0048</t>
+          <t>PWD-LB-2024-0043</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1775,42 +1613,36 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0.1</v>
+        <v>0.75</v>
       </c>
       <c r="D23" t="n">
-        <v>0.21</v>
+        <v>0.91</v>
       </c>
       <c r="E23" t="n">
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G23" t="n">
         <v>1</v>
       </c>
       <c r="H23" t="n">
-        <v>0</v>
-      </c>
-      <c r="I23" t="n">
-        <v>1</v>
-      </c>
-      <c r="J23" t="n">
-        <v>1</v>
-      </c>
-      <c r="K23" t="b">
+        <v>1</v>
+      </c>
+      <c r="I23" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>PWD-LB-2024-0046</t>
+          <t>PWD-LB-2024-0045</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>JOB-002</t>
+          <t>JOB-001</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -1823,21 +1655,15 @@
         <v>0.3</v>
       </c>
       <c r="F24" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H24" t="n">
         <v>0</v>
       </c>
-      <c r="I24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K24" t="b">
+      <c r="I24" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1852,7 +1678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K92"/>
+  <dimension ref="A1:I92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1883,30 +1709,20 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>location_fraction</t>
+          <t>disability_listed</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>preference_fraction</t>
+          <t>label</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>disability_listed</t>
+          <t>label_gated</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>label</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>label_gated</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>score</t>
         </is>
@@ -1933,22 +1749,16 @@
         <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
         <v>1</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K2" t="n">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3">
@@ -1972,22 +1782,16 @@
         <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
         <v>1</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J3" t="n">
-        <v>1</v>
-      </c>
-      <c r="K3" t="n">
-        <v>63</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4">
@@ -2011,7 +1815,7 @@
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G4" t="n">
         <v>1</v>
@@ -2020,13 +1824,7 @@
         <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="n">
-        <v>75</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5">
@@ -2050,22 +1848,16 @@
         <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
-      </c>
-      <c r="J5" t="n">
-        <v>1</v>
-      </c>
-      <c r="K5" t="n">
-        <v>71</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6">
@@ -2089,22 +1881,16 @@
         <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>0.35</v>
+        <v>0</v>
       </c>
       <c r="G6" t="n">
         <v>1</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I6" t="n">
-        <v>1</v>
-      </c>
-      <c r="J6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K6" t="n">
-        <v>77</v>
+        <v>82</v>
       </c>
     </row>
     <row r="7">
@@ -2128,22 +1914,16 @@
         <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>0.35</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
         <v>1</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J7" t="n">
-        <v>1</v>
-      </c>
-      <c r="K7" t="n">
-        <v>72</v>
+        <v>75</v>
       </c>
     </row>
     <row r="8">
@@ -2167,22 +1947,16 @@
         <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G8" t="n">
         <v>1</v>
       </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I8" t="n">
-        <v>1</v>
-      </c>
-      <c r="J8" t="n">
-        <v>1</v>
-      </c>
-      <c r="K8" t="n">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="9">
@@ -2206,22 +1980,16 @@
         <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>1</v>
-      </c>
-      <c r="J9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" t="n">
-        <v>42</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10">
@@ -2245,22 +2013,16 @@
         <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H10" t="n">
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>1</v>
-      </c>
-      <c r="J10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" t="n">
-        <v>41</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11">
@@ -2284,22 +2046,16 @@
         <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>1</v>
-      </c>
-      <c r="J11" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" t="n">
-        <v>41</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12">
@@ -2323,22 +2079,16 @@
         <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>1</v>
-      </c>
-      <c r="J12" t="n">
-        <v>0</v>
-      </c>
-      <c r="K12" t="n">
-        <v>47</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13">
@@ -2362,22 +2112,16 @@
         <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" t="n">
-        <v>36</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14">
@@ -2401,22 +2145,16 @@
         <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
       </c>
       <c r="I14" t="n">
-        <v>1</v>
-      </c>
-      <c r="J14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K14" t="n">
-        <v>46</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15">
@@ -2440,21 +2178,15 @@
         <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G15" t="n">
         <v>1</v>
       </c>
       <c r="H15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I15" t="n">
-        <v>1</v>
-      </c>
-      <c r="J15" t="n">
-        <v>1</v>
-      </c>
-      <c r="K15" t="n">
         <v>85</v>
       </c>
     </row>
@@ -2479,22 +2211,16 @@
         <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G16" t="n">
         <v>1</v>
       </c>
       <c r="H16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I16" t="n">
-        <v>1</v>
-      </c>
-      <c r="J16" t="n">
-        <v>1</v>
-      </c>
-      <c r="K16" t="n">
-        <v>80</v>
+        <v>73</v>
       </c>
     </row>
     <row r="17">
@@ -2518,22 +2244,16 @@
         <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>1</v>
-      </c>
-      <c r="J17" t="n">
-        <v>0</v>
-      </c>
-      <c r="K17" t="n">
-        <v>58</v>
+        <v>50</v>
       </c>
     </row>
     <row r="18">
@@ -2557,22 +2277,16 @@
         <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I18" t="n">
-        <v>1</v>
-      </c>
-      <c r="J18" t="n">
-        <v>1</v>
-      </c>
-      <c r="K18" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
     </row>
     <row r="19">
@@ -2596,7 +2310,7 @@
         <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>0.35</v>
+        <v>0</v>
       </c>
       <c r="G19" t="n">
         <v>1</v>
@@ -2605,12 +2319,6 @@
         <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>1</v>
-      </c>
-      <c r="J19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K19" t="n">
         <v>62</v>
       </c>
     </row>
@@ -2635,7 +2343,7 @@
         <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>0.35</v>
+        <v>0</v>
       </c>
       <c r="G20" t="n">
         <v>1</v>
@@ -2644,12 +2352,6 @@
         <v>0</v>
       </c>
       <c r="I20" t="n">
-        <v>1</v>
-      </c>
-      <c r="J20" t="n">
-        <v>0</v>
-      </c>
-      <c r="K20" t="n">
         <v>62</v>
       </c>
     </row>
@@ -2674,22 +2376,16 @@
         <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G21" t="n">
         <v>1</v>
       </c>
       <c r="H21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I21" t="n">
-        <v>1</v>
-      </c>
-      <c r="J21" t="n">
-        <v>1</v>
-      </c>
-      <c r="K21" t="n">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="22">
@@ -2713,7 +2409,7 @@
         <v>1</v>
       </c>
       <c r="F22" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G22" t="n">
         <v>0</v>
@@ -2722,13 +2418,7 @@
         <v>0</v>
       </c>
       <c r="I22" t="n">
-        <v>0</v>
-      </c>
-      <c r="J22" t="n">
-        <v>0</v>
-      </c>
-      <c r="K22" t="n">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="23">
@@ -2752,22 +2442,16 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H23" t="n">
         <v>0</v>
       </c>
       <c r="I23" t="n">
-        <v>1</v>
-      </c>
-      <c r="J23" t="n">
-        <v>0</v>
-      </c>
-      <c r="K23" t="n">
-        <v>45</v>
+        <v>27</v>
       </c>
     </row>
     <row r="24">
@@ -2791,22 +2475,16 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H24" t="n">
         <v>0</v>
       </c>
       <c r="I24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K24" t="n">
-        <v>36</v>
+        <v>27</v>
       </c>
     </row>
     <row r="25">
@@ -2830,7 +2508,7 @@
         <v>1</v>
       </c>
       <c r="F25" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G25" t="n">
         <v>1</v>
@@ -2839,13 +2517,7 @@
         <v>0</v>
       </c>
       <c r="I25" t="n">
-        <v>1</v>
-      </c>
-      <c r="J25" t="n">
-        <v>0</v>
-      </c>
-      <c r="K25" t="n">
-        <v>58</v>
+        <v>50</v>
       </c>
     </row>
     <row r="26">
@@ -2869,22 +2541,16 @@
         <v>1</v>
       </c>
       <c r="F26" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G26" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H26" t="n">
         <v>0</v>
       </c>
       <c r="I26" t="n">
-        <v>0</v>
-      </c>
-      <c r="J26" t="n">
-        <v>0</v>
-      </c>
-      <c r="K26" t="n">
-        <v>36</v>
+        <v>27</v>
       </c>
     </row>
     <row r="27">
@@ -2908,22 +2574,16 @@
         <v>1</v>
       </c>
       <c r="F27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H27" t="n">
         <v>0</v>
       </c>
       <c r="I27" t="n">
-        <v>1</v>
-      </c>
-      <c r="J27" t="n">
-        <v>0</v>
-      </c>
-      <c r="K27" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="28">
@@ -2947,22 +2607,16 @@
         <v>1</v>
       </c>
       <c r="F28" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G28" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H28" t="n">
         <v>0</v>
       </c>
       <c r="I28" t="n">
-        <v>0</v>
-      </c>
-      <c r="J28" t="n">
-        <v>0</v>
-      </c>
-      <c r="K28" t="n">
-        <v>36</v>
+        <v>27</v>
       </c>
     </row>
     <row r="29">
@@ -2986,22 +2640,16 @@
         <v>1</v>
       </c>
       <c r="F29" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G29" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H29" t="n">
         <v>0</v>
       </c>
       <c r="I29" t="n">
-        <v>0</v>
-      </c>
-      <c r="J29" t="n">
-        <v>0</v>
-      </c>
-      <c r="K29" t="n">
-        <v>36</v>
+        <v>27</v>
       </c>
     </row>
     <row r="30">
@@ -3025,22 +2673,16 @@
         <v>1</v>
       </c>
       <c r="F30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G30" t="n">
         <v>1</v>
       </c>
       <c r="H30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I30" t="n">
-        <v>1</v>
-      </c>
-      <c r="J30" t="n">
-        <v>1</v>
-      </c>
-      <c r="K30" t="n">
-        <v>61</v>
+        <v>48</v>
       </c>
     </row>
     <row r="31">
@@ -3064,22 +2706,16 @@
         <v>1</v>
       </c>
       <c r="F31" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H31" t="n">
         <v>0</v>
       </c>
       <c r="I31" t="n">
-        <v>1</v>
-      </c>
-      <c r="J31" t="n">
-        <v>0</v>
-      </c>
-      <c r="K31" t="n">
-        <v>41</v>
+        <v>27</v>
       </c>
     </row>
     <row r="32">
@@ -3103,22 +2739,16 @@
         <v>1</v>
       </c>
       <c r="F32" t="n">
-        <v>0.35</v>
+        <v>0</v>
       </c>
       <c r="G32" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H32" t="n">
         <v>0</v>
       </c>
       <c r="I32" t="n">
-        <v>0</v>
-      </c>
-      <c r="J32" t="n">
-        <v>0</v>
-      </c>
-      <c r="K32" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="33">
@@ -3142,22 +2772,16 @@
         <v>1</v>
       </c>
       <c r="F33" t="n">
-        <v>0.35</v>
+        <v>0</v>
       </c>
       <c r="G33" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H33" t="n">
         <v>0</v>
       </c>
       <c r="I33" t="n">
-        <v>0</v>
-      </c>
-      <c r="J33" t="n">
-        <v>0</v>
-      </c>
-      <c r="K33" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="34">
@@ -3181,22 +2805,16 @@
         <v>1</v>
       </c>
       <c r="F34" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G34" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H34" t="n">
         <v>0</v>
       </c>
       <c r="I34" t="n">
-        <v>0</v>
-      </c>
-      <c r="J34" t="n">
-        <v>0</v>
-      </c>
-      <c r="K34" t="n">
-        <v>36</v>
+        <v>27</v>
       </c>
     </row>
     <row r="35">
@@ -3220,22 +2838,16 @@
         <v>1</v>
       </c>
       <c r="F35" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G35" t="n">
         <v>1</v>
       </c>
       <c r="H35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I35" t="n">
-        <v>1</v>
-      </c>
-      <c r="J35" t="n">
-        <v>1</v>
-      </c>
-      <c r="K35" t="n">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="36">
@@ -3259,22 +2871,16 @@
         <v>1</v>
       </c>
       <c r="F36" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G36" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H36" t="n">
         <v>0</v>
       </c>
       <c r="I36" t="n">
-        <v>1</v>
-      </c>
-      <c r="J36" t="n">
-        <v>0</v>
-      </c>
-      <c r="K36" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
     </row>
     <row r="37">
@@ -3298,22 +2904,16 @@
         <v>1</v>
       </c>
       <c r="F37" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G37" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H37" t="n">
         <v>0</v>
       </c>
       <c r="I37" t="n">
-        <v>1</v>
-      </c>
-      <c r="J37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K37" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
     </row>
     <row r="38">
@@ -3337,22 +2937,16 @@
         <v>1</v>
       </c>
       <c r="F38" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G38" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H38" t="n">
         <v>0</v>
       </c>
       <c r="I38" t="n">
-        <v>0</v>
-      </c>
-      <c r="J38" t="n">
-        <v>0</v>
-      </c>
-      <c r="K38" t="n">
-        <v>36</v>
+        <v>27</v>
       </c>
     </row>
     <row r="39">
@@ -3376,7 +2970,7 @@
         <v>1</v>
       </c>
       <c r="F39" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G39" t="n">
         <v>0</v>
@@ -3385,13 +2979,7 @@
         <v>0</v>
       </c>
       <c r="I39" t="n">
-        <v>1</v>
-      </c>
-      <c r="J39" t="n">
-        <v>0</v>
-      </c>
-      <c r="K39" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="40">
@@ -3415,22 +3003,16 @@
         <v>1</v>
       </c>
       <c r="F40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G40" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I40" t="n">
-        <v>1</v>
-      </c>
-      <c r="J40" t="n">
-        <v>1</v>
-      </c>
-      <c r="K40" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="41">
@@ -3454,22 +3036,16 @@
         <v>0.3</v>
       </c>
       <c r="F41" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H41" t="n">
         <v>0</v>
       </c>
       <c r="I41" t="n">
-        <v>0</v>
-      </c>
-      <c r="J41" t="n">
-        <v>0</v>
-      </c>
-      <c r="K41" t="n">
-        <v>30</v>
+        <v>13</v>
       </c>
     </row>
     <row r="42">
@@ -3493,22 +3069,16 @@
         <v>0.1</v>
       </c>
       <c r="F42" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G42" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H42" t="n">
         <v>0</v>
       </c>
       <c r="I42" t="n">
-        <v>0</v>
-      </c>
-      <c r="J42" t="n">
-        <v>0</v>
-      </c>
-      <c r="K42" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
     </row>
     <row r="43">
@@ -3532,22 +3102,16 @@
         <v>0.1</v>
       </c>
       <c r="F43" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G43" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H43" t="n">
         <v>0</v>
       </c>
       <c r="I43" t="n">
-        <v>0</v>
-      </c>
-      <c r="J43" t="n">
-        <v>0</v>
-      </c>
-      <c r="K43" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
     </row>
     <row r="44">
@@ -3571,22 +3135,16 @@
         <v>0.1</v>
       </c>
       <c r="F44" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G44" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H44" t="n">
         <v>0</v>
       </c>
       <c r="I44" t="n">
-        <v>0</v>
-      </c>
-      <c r="J44" t="n">
-        <v>0</v>
-      </c>
-      <c r="K44" t="n">
-        <v>22</v>
+        <v>9</v>
       </c>
     </row>
     <row r="45">
@@ -3610,22 +3168,16 @@
         <v>0.3</v>
       </c>
       <c r="F45" t="n">
-        <v>0.35</v>
+        <v>0</v>
       </c>
       <c r="G45" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H45" t="n">
         <v>0</v>
       </c>
       <c r="I45" t="n">
-        <v>0</v>
-      </c>
-      <c r="J45" t="n">
-        <v>0</v>
-      </c>
-      <c r="K45" t="n">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="46">
@@ -3649,22 +3201,16 @@
         <v>1</v>
       </c>
       <c r="F46" t="n">
-        <v>0.35</v>
+        <v>0</v>
       </c>
       <c r="G46" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H46" t="n">
         <v>0</v>
       </c>
       <c r="I46" t="n">
-        <v>0</v>
-      </c>
-      <c r="J46" t="n">
-        <v>0</v>
-      </c>
-      <c r="K46" t="n">
-        <v>36</v>
+        <v>27</v>
       </c>
     </row>
     <row r="47">
@@ -3688,22 +3234,16 @@
         <v>0.1</v>
       </c>
       <c r="F47" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H47" t="n">
         <v>0</v>
       </c>
       <c r="I47" t="n">
-        <v>0</v>
-      </c>
-      <c r="J47" t="n">
-        <v>0</v>
-      </c>
-      <c r="K47" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
     </row>
     <row r="48">
@@ -3727,7 +3267,7 @@
         <v>0.3</v>
       </c>
       <c r="F48" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G48" t="n">
         <v>0</v>
@@ -3736,13 +3276,7 @@
         <v>0</v>
       </c>
       <c r="I48" t="n">
-        <v>0</v>
-      </c>
-      <c r="J48" t="n">
-        <v>0</v>
-      </c>
-      <c r="K48" t="n">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="49">
@@ -3766,22 +3300,16 @@
         <v>1</v>
       </c>
       <c r="F49" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G49" t="n">
         <v>1</v>
       </c>
       <c r="H49" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I49" t="n">
-        <v>1</v>
-      </c>
-      <c r="J49" t="n">
-        <v>1</v>
-      </c>
-      <c r="K49" t="n">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="50">
@@ -3805,22 +3333,16 @@
         <v>1</v>
       </c>
       <c r="F50" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G50" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H50" t="n">
         <v>0</v>
       </c>
       <c r="I50" t="n">
-        <v>1</v>
-      </c>
-      <c r="J50" t="n">
-        <v>0</v>
-      </c>
-      <c r="K50" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="51">
@@ -3844,22 +3366,16 @@
         <v>1</v>
       </c>
       <c r="F51" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G51" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H51" t="n">
         <v>0</v>
       </c>
       <c r="I51" t="n">
-        <v>1</v>
-      </c>
-      <c r="J51" t="n">
-        <v>0</v>
-      </c>
-      <c r="K51" t="n">
-        <v>50</v>
+        <v>38</v>
       </c>
     </row>
     <row r="52">
@@ -3883,22 +3399,16 @@
         <v>1</v>
       </c>
       <c r="F52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G52" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I52" t="n">
-        <v>1</v>
-      </c>
-      <c r="J52" t="n">
-        <v>1</v>
-      </c>
-      <c r="K52" t="n">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="53">
@@ -3922,22 +3432,16 @@
         <v>0.6</v>
       </c>
       <c r="F53" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G53" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H53" t="n">
         <v>0</v>
       </c>
       <c r="I53" t="n">
-        <v>1</v>
-      </c>
-      <c r="J53" t="n">
-        <v>0</v>
-      </c>
-      <c r="K53" t="n">
-        <v>47</v>
+        <v>42</v>
       </c>
     </row>
     <row r="54">
@@ -3961,22 +3465,16 @@
         <v>1</v>
       </c>
       <c r="F54" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G54" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H54" t="n">
         <v>0</v>
       </c>
       <c r="I54" t="n">
-        <v>0</v>
-      </c>
-      <c r="J54" t="n">
-        <v>0</v>
-      </c>
-      <c r="K54" t="n">
-        <v>36</v>
+        <v>27</v>
       </c>
     </row>
     <row r="55">
@@ -4000,22 +3498,16 @@
         <v>0.3</v>
       </c>
       <c r="F55" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G55" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H55" t="n">
         <v>0</v>
       </c>
       <c r="I55" t="n">
-        <v>0</v>
-      </c>
-      <c r="J55" t="n">
-        <v>0</v>
-      </c>
-      <c r="K55" t="n">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="56">
@@ -4039,7 +3531,7 @@
         <v>0.3</v>
       </c>
       <c r="F56" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G56" t="n">
         <v>0</v>
@@ -4048,13 +3540,7 @@
         <v>0</v>
       </c>
       <c r="I56" t="n">
-        <v>1</v>
-      </c>
-      <c r="J56" t="n">
-        <v>0</v>
-      </c>
-      <c r="K56" t="n">
-        <v>42</v>
+        <v>36</v>
       </c>
     </row>
     <row r="57">
@@ -4078,7 +3564,7 @@
         <v>0.3</v>
       </c>
       <c r="F57" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G57" t="n">
         <v>0</v>
@@ -4087,13 +3573,7 @@
         <v>0</v>
       </c>
       <c r="I57" t="n">
-        <v>0</v>
-      </c>
-      <c r="J57" t="n">
-        <v>0</v>
-      </c>
-      <c r="K57" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
     </row>
     <row r="58">
@@ -4117,22 +3597,16 @@
         <v>1</v>
       </c>
       <c r="F58" t="n">
-        <v>0.35</v>
+        <v>0</v>
       </c>
       <c r="G58" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H58" t="n">
         <v>0</v>
       </c>
       <c r="I58" t="n">
-        <v>0</v>
-      </c>
-      <c r="J58" t="n">
-        <v>0</v>
-      </c>
-      <c r="K58" t="n">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="59">
@@ -4156,22 +3630,16 @@
         <v>1</v>
       </c>
       <c r="F59" t="n">
-        <v>0.35</v>
+        <v>0</v>
       </c>
       <c r="G59" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H59" t="n">
         <v>0</v>
       </c>
       <c r="I59" t="n">
-        <v>0</v>
-      </c>
-      <c r="J59" t="n">
-        <v>0</v>
-      </c>
-      <c r="K59" t="n">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="60">
@@ -4195,22 +3663,16 @@
         <v>0.3</v>
       </c>
       <c r="F60" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G60" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H60" t="n">
         <v>0</v>
       </c>
       <c r="I60" t="n">
-        <v>0</v>
-      </c>
-      <c r="J60" t="n">
-        <v>0</v>
-      </c>
-      <c r="K60" t="n">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="61">
@@ -4234,22 +3696,16 @@
         <v>1</v>
       </c>
       <c r="F61" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G61" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H61" t="n">
         <v>0</v>
       </c>
       <c r="I61" t="n">
-        <v>1</v>
-      </c>
-      <c r="J61" t="n">
-        <v>0</v>
-      </c>
-      <c r="K61" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="62">
@@ -4273,22 +3729,16 @@
         <v>1</v>
       </c>
       <c r="F62" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G62" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H62" t="n">
         <v>0</v>
       </c>
       <c r="I62" t="n">
-        <v>1</v>
-      </c>
-      <c r="J62" t="n">
-        <v>0</v>
-      </c>
-      <c r="K62" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="63">
@@ -4312,22 +3762,16 @@
         <v>1</v>
       </c>
       <c r="F63" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G63" t="n">
         <v>1</v>
       </c>
       <c r="H63" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I63" t="n">
-        <v>1</v>
-      </c>
-      <c r="J63" t="n">
-        <v>1</v>
-      </c>
-      <c r="K63" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="64">
@@ -4351,22 +3795,16 @@
         <v>1</v>
       </c>
       <c r="F64" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G64" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H64" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I64" t="n">
-        <v>1</v>
-      </c>
-      <c r="J64" t="n">
-        <v>1</v>
-      </c>
-      <c r="K64" t="n">
-        <v>88</v>
+        <v>97</v>
       </c>
     </row>
     <row r="65">
@@ -4390,22 +3828,16 @@
         <v>1</v>
       </c>
       <c r="F65" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G65" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H65" t="n">
         <v>0</v>
       </c>
       <c r="I65" t="n">
-        <v>1</v>
-      </c>
-      <c r="J65" t="n">
-        <v>0</v>
-      </c>
-      <c r="K65" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="66">
@@ -4429,22 +3861,16 @@
         <v>1</v>
       </c>
       <c r="F66" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G66" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H66" t="n">
         <v>0</v>
       </c>
       <c r="I66" t="n">
-        <v>1</v>
-      </c>
-      <c r="J66" t="n">
-        <v>0</v>
-      </c>
-      <c r="K66" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="67">
@@ -4468,22 +3894,16 @@
         <v>0.6</v>
       </c>
       <c r="F67" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G67" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H67" t="n">
         <v>0</v>
       </c>
       <c r="I67" t="n">
-        <v>0</v>
-      </c>
-      <c r="J67" t="n">
-        <v>0</v>
-      </c>
-      <c r="K67" t="n">
-        <v>30</v>
+        <v>19</v>
       </c>
     </row>
     <row r="68">
@@ -4507,22 +3927,16 @@
         <v>0.1</v>
       </c>
       <c r="F68" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G68" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H68" t="n">
         <v>0</v>
       </c>
       <c r="I68" t="n">
-        <v>0</v>
-      </c>
-      <c r="J68" t="n">
-        <v>0</v>
-      </c>
-      <c r="K68" t="n">
-        <v>22</v>
+        <v>9</v>
       </c>
     </row>
     <row r="69">
@@ -4546,22 +3960,16 @@
         <v>0.1</v>
       </c>
       <c r="F69" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G69" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H69" t="n">
         <v>0</v>
       </c>
       <c r="I69" t="n">
-        <v>0</v>
-      </c>
-      <c r="J69" t="n">
-        <v>0</v>
-      </c>
-      <c r="K69" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
     </row>
     <row r="70">
@@ -4585,7 +3993,7 @@
         <v>0.1</v>
       </c>
       <c r="F70" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G70" t="n">
         <v>0</v>
@@ -4594,13 +4002,7 @@
         <v>0</v>
       </c>
       <c r="I70" t="n">
-        <v>0</v>
-      </c>
-      <c r="J70" t="n">
-        <v>0</v>
-      </c>
-      <c r="K70" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
     </row>
     <row r="71">
@@ -4624,22 +4026,16 @@
         <v>0.6</v>
       </c>
       <c r="F71" t="n">
-        <v>0.35</v>
+        <v>0</v>
       </c>
       <c r="G71" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H71" t="n">
         <v>0</v>
       </c>
       <c r="I71" t="n">
-        <v>0</v>
-      </c>
-      <c r="J71" t="n">
-        <v>0</v>
-      </c>
-      <c r="K71" t="n">
-        <v>25</v>
+        <v>19</v>
       </c>
     </row>
     <row r="72">
@@ -4663,22 +4059,16 @@
         <v>1</v>
       </c>
       <c r="F72" t="n">
-        <v>0.35</v>
+        <v>0</v>
       </c>
       <c r="G72" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H72" t="n">
         <v>0</v>
       </c>
       <c r="I72" t="n">
-        <v>0</v>
-      </c>
-      <c r="J72" t="n">
-        <v>0</v>
-      </c>
-      <c r="K72" t="n">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="73">
@@ -4702,22 +4092,16 @@
         <v>0.1</v>
       </c>
       <c r="F73" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G73" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H73" t="n">
         <v>0</v>
       </c>
       <c r="I73" t="n">
-        <v>0</v>
-      </c>
-      <c r="J73" t="n">
-        <v>0</v>
-      </c>
-      <c r="K73" t="n">
-        <v>22</v>
+        <v>9</v>
       </c>
     </row>
     <row r="74">
@@ -4741,22 +4125,16 @@
         <v>0.6</v>
       </c>
       <c r="F74" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G74" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H74" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I74" t="n">
-        <v>1</v>
-      </c>
-      <c r="J74" t="n">
-        <v>1</v>
-      </c>
-      <c r="K74" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="75">
@@ -4780,22 +4158,16 @@
         <v>1</v>
       </c>
       <c r="F75" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G75" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H75" t="n">
         <v>0</v>
       </c>
       <c r="I75" t="n">
-        <v>1</v>
-      </c>
-      <c r="J75" t="n">
-        <v>0</v>
-      </c>
-      <c r="K75" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="76">
@@ -4819,7 +4191,7 @@
         <v>1</v>
       </c>
       <c r="F76" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G76" t="n">
         <v>1</v>
@@ -4828,13 +4200,7 @@
         <v>0</v>
       </c>
       <c r="I76" t="n">
-        <v>1</v>
-      </c>
-      <c r="J76" t="n">
-        <v>0</v>
-      </c>
-      <c r="K76" t="n">
-        <v>58</v>
+        <v>50</v>
       </c>
     </row>
     <row r="77">
@@ -4858,22 +4224,16 @@
         <v>1</v>
       </c>
       <c r="F77" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G77" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H77" t="n">
         <v>0</v>
       </c>
       <c r="I77" t="n">
-        <v>0</v>
-      </c>
-      <c r="J77" t="n">
-        <v>0</v>
-      </c>
-      <c r="K77" t="n">
-        <v>36</v>
+        <v>27</v>
       </c>
     </row>
     <row r="78">
@@ -4897,7 +4257,7 @@
         <v>1</v>
       </c>
       <c r="F78" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G78" t="n">
         <v>1</v>
@@ -4906,13 +4266,7 @@
         <v>0</v>
       </c>
       <c r="I78" t="n">
-        <v>1</v>
-      </c>
-      <c r="J78" t="n">
-        <v>0</v>
-      </c>
-      <c r="K78" t="n">
-        <v>58</v>
+        <v>50</v>
       </c>
     </row>
     <row r="79">
@@ -4936,22 +4290,16 @@
         <v>1</v>
       </c>
       <c r="F79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G79" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I79" t="n">
-        <v>1</v>
-      </c>
-      <c r="J79" t="n">
-        <v>1</v>
-      </c>
-      <c r="K79" t="n">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="80">
@@ -4975,22 +4323,16 @@
         <v>1</v>
       </c>
       <c r="F80" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G80" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H80" t="n">
         <v>0</v>
       </c>
       <c r="I80" t="n">
-        <v>1</v>
-      </c>
-      <c r="J80" t="n">
-        <v>0</v>
-      </c>
-      <c r="K80" t="n">
-        <v>44</v>
+        <v>32</v>
       </c>
     </row>
     <row r="81">
@@ -5014,22 +4356,16 @@
         <v>1</v>
       </c>
       <c r="F81" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G81" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H81" t="n">
         <v>0</v>
       </c>
       <c r="I81" t="n">
-        <v>1</v>
-      </c>
-      <c r="J81" t="n">
-        <v>0</v>
-      </c>
-      <c r="K81" t="n">
-        <v>41</v>
+        <v>27</v>
       </c>
     </row>
     <row r="82">
@@ -5053,22 +4389,16 @@
         <v>1</v>
       </c>
       <c r="F82" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G82" t="n">
         <v>1</v>
       </c>
       <c r="H82" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I82" t="n">
-        <v>1</v>
-      </c>
-      <c r="J82" t="n">
-        <v>1</v>
-      </c>
-      <c r="K82" t="n">
-        <v>75</v>
+        <v>67</v>
       </c>
     </row>
     <row r="83">
@@ -5092,22 +4422,16 @@
         <v>1</v>
       </c>
       <c r="F83" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G83" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H83" t="n">
         <v>0</v>
       </c>
       <c r="I83" t="n">
-        <v>1</v>
-      </c>
-      <c r="J83" t="n">
-        <v>0</v>
-      </c>
-      <c r="K83" t="n">
-        <v>45</v>
+        <v>39</v>
       </c>
     </row>
     <row r="84">
@@ -5131,21 +4455,15 @@
         <v>1</v>
       </c>
       <c r="F84" t="n">
-        <v>0.35</v>
+        <v>0</v>
       </c>
       <c r="G84" t="n">
         <v>1</v>
       </c>
       <c r="H84" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I84" t="n">
-        <v>1</v>
-      </c>
-      <c r="J84" t="n">
-        <v>1</v>
-      </c>
-      <c r="K84" t="n">
         <v>62</v>
       </c>
     </row>
@@ -5170,22 +4488,16 @@
         <v>1</v>
       </c>
       <c r="F85" t="n">
-        <v>0.35</v>
+        <v>0</v>
       </c>
       <c r="G85" t="n">
         <v>1</v>
       </c>
       <c r="H85" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I85" t="n">
-        <v>1</v>
-      </c>
-      <c r="J85" t="n">
-        <v>1</v>
-      </c>
-      <c r="K85" t="n">
-        <v>71</v>
+        <v>74</v>
       </c>
     </row>
     <row r="86">
@@ -5209,22 +4521,16 @@
         <v>1</v>
       </c>
       <c r="F86" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G86" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H86" t="n">
         <v>0</v>
       </c>
       <c r="I86" t="n">
-        <v>1</v>
-      </c>
-      <c r="J86" t="n">
-        <v>0</v>
-      </c>
-      <c r="K86" t="n">
-        <v>44</v>
+        <v>31</v>
       </c>
     </row>
     <row r="87">
@@ -5248,22 +4554,16 @@
         <v>1</v>
       </c>
       <c r="F87" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G87" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H87" t="n">
         <v>0</v>
       </c>
       <c r="I87" t="n">
-        <v>1</v>
-      </c>
-      <c r="J87" t="n">
-        <v>0</v>
-      </c>
-      <c r="K87" t="n">
-        <v>48</v>
+        <v>43</v>
       </c>
     </row>
     <row r="88">
@@ -5287,22 +4587,16 @@
         <v>1</v>
       </c>
       <c r="F88" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G88" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H88" t="n">
         <v>0</v>
       </c>
       <c r="I88" t="n">
-        <v>1</v>
-      </c>
-      <c r="J88" t="n">
-        <v>0</v>
-      </c>
-      <c r="K88" t="n">
-        <v>50</v>
+        <v>38</v>
       </c>
     </row>
     <row r="89">
@@ -5326,22 +4620,16 @@
         <v>1</v>
       </c>
       <c r="F89" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G89" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H89" t="n">
         <v>0</v>
       </c>
       <c r="I89" t="n">
-        <v>1</v>
-      </c>
-      <c r="J89" t="n">
-        <v>0</v>
-      </c>
-      <c r="K89" t="n">
-        <v>50</v>
+        <v>38</v>
       </c>
     </row>
     <row r="90">
@@ -5365,22 +4653,16 @@
         <v>1</v>
       </c>
       <c r="F90" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G90" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H90" t="n">
         <v>0</v>
       </c>
       <c r="I90" t="n">
-        <v>1</v>
-      </c>
-      <c r="J90" t="n">
-        <v>0</v>
-      </c>
-      <c r="K90" t="n">
-        <v>50</v>
+        <v>38</v>
       </c>
     </row>
     <row r="91">
@@ -5404,22 +4686,16 @@
         <v>1</v>
       </c>
       <c r="F91" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G91" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H91" t="n">
         <v>0</v>
       </c>
       <c r="I91" t="n">
-        <v>1</v>
-      </c>
-      <c r="J91" t="n">
-        <v>0</v>
-      </c>
-      <c r="K91" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
     </row>
     <row r="92">
@@ -5443,22 +4719,16 @@
         <v>1</v>
       </c>
       <c r="F92" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G92" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H92" t="n">
         <v>0</v>
       </c>
       <c r="I92" t="n">
-        <v>1</v>
-      </c>
-      <c r="J92" t="n">
-        <v>0</v>
-      </c>
-      <c r="K92" t="n">
-        <v>49</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>